<commit_message>
chg: Updated admin instructions with change from OvGME to Open Mod Manager
</commit_message>
<xml_diff>
--- a/COMMUNICATIONS/OPAC Frequency and callsign master list.xlsx
+++ b/COMMUNICATIONS/OPAC Frequency and callsign master list.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
   </bookViews>
   <sheets>
     <sheet name="Frequencies" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2330" uniqueCount="1350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="1352">
   <si>
     <t>AWACS</t>
   </si>
@@ -4075,6 +4075,12 @@
   </si>
   <si>
     <t>BANSHEE 3</t>
+  </si>
+  <si>
+    <t>MADRID</t>
+  </si>
+  <si>
+    <t>126.35</t>
   </si>
 </sst>
 </file>
@@ -6803,12 +6809,21 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6818,14 +6833,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6836,6 +6845,9 @@
     <xf numFmtId="0" fontId="24" fillId="18" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6863,12 +6875,6 @@
     <xf numFmtId="0" fontId="25" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6938,6 +6944,54 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="102" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="100" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="101" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="50" fillId="8" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="50" fillId="8" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6995,54 +7049,6 @@
     <xf numFmtId="49" fontId="41" fillId="31" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="39" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="39" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="39" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="39" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="102" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="100" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="101" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="50" fillId="8" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -7151,6 +7157,57 @@
     <xf numFmtId="0" fontId="31" fillId="20" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="8" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="8" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="8" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="13" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="13" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7168,57 +7225,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="13" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="13" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="13" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="8" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="8" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="8" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -7650,13 +7656,13 @@
       <c r="N2" s="105" t="s">
         <v>329</v>
       </c>
-      <c r="V2" s="334" t="s">
+      <c r="V2" s="333" t="s">
         <v>0</v>
       </c>
-      <c r="W2" s="334"/>
-      <c r="X2" s="334"/>
-      <c r="Y2" s="334"/>
-      <c r="Z2" s="334"/>
+      <c r="W2" s="333"/>
+      <c r="X2" s="333"/>
+      <c r="Y2" s="333"/>
+      <c r="Z2" s="333"/>
     </row>
     <row r="3" spans="1:42">
       <c r="A3" s="105" t="s">
@@ -7705,9 +7711,9 @@
       <c r="P3" t="s">
         <v>425</v>
       </c>
-      <c r="R3" s="333"/>
-      <c r="S3" s="333"/>
-      <c r="T3" s="333"/>
+      <c r="R3" s="337"/>
+      <c r="S3" s="337"/>
+      <c r="T3" s="337"/>
       <c r="V3" s="99" t="s">
         <v>328</v>
       </c>
@@ -7789,22 +7795,22 @@
       <c r="AA4" s="21"/>
       <c r="AB4" s="21"/>
       <c r="AC4" s="21"/>
-      <c r="AD4" s="334" t="s">
+      <c r="AD4" s="333" t="s">
         <v>428</v>
       </c>
-      <c r="AE4" s="334"/>
-      <c r="AF4" s="334"/>
-      <c r="AG4" s="334"/>
-      <c r="AH4" s="334"/>
-      <c r="AJ4" s="334" t="s">
+      <c r="AE4" s="333"/>
+      <c r="AF4" s="333"/>
+      <c r="AG4" s="333"/>
+      <c r="AH4" s="333"/>
+      <c r="AJ4" s="333" t="s">
         <v>1</v>
       </c>
-      <c r="AK4" s="334"/>
-      <c r="AL4" s="334"/>
-      <c r="AM4" s="334"/>
-      <c r="AN4" s="334"/>
-      <c r="AO4" s="334"/>
-      <c r="AP4" s="334"/>
+      <c r="AK4" s="333"/>
+      <c r="AL4" s="333"/>
+      <c r="AM4" s="333"/>
+      <c r="AN4" s="333"/>
+      <c r="AO4" s="333"/>
+      <c r="AP4" s="333"/>
     </row>
     <row r="5" spans="1:42" ht="15.75">
       <c r="A5" s="105" t="s">
@@ -8993,15 +8999,15 @@
       <c r="AH18" s="3" t="s">
         <v>471</v>
       </c>
-      <c r="AJ18" s="334" t="s">
+      <c r="AJ18" s="333" t="s">
         <v>274</v>
       </c>
-      <c r="AK18" s="334"/>
-      <c r="AL18" s="334"/>
-      <c r="AM18" s="334"/>
-      <c r="AN18" s="334"/>
-      <c r="AO18" s="334"/>
-      <c r="AP18" s="334"/>
+      <c r="AK18" s="333"/>
+      <c r="AL18" s="333"/>
+      <c r="AM18" s="333"/>
+      <c r="AN18" s="333"/>
+      <c r="AO18" s="333"/>
+      <c r="AP18" s="333"/>
     </row>
     <row r="19" spans="1:42" ht="15.75">
       <c r="A19" s="105" t="s">
@@ -9134,9 +9140,9 @@
       </c>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
-      <c r="R20" s="333"/>
-      <c r="S20" s="333"/>
-      <c r="T20" s="333"/>
+      <c r="R20" s="337"/>
+      <c r="S20" s="337"/>
+      <c r="T20" s="337"/>
       <c r="U20" s="2"/>
       <c r="V20" s="224" t="s">
         <v>1126</v>
@@ -9531,13 +9537,13 @@
       <c r="R25" s="22"/>
       <c r="S25" s="22"/>
       <c r="T25" s="22"/>
-      <c r="AD25" s="334" t="s">
+      <c r="AD25" s="333" t="s">
         <v>485</v>
       </c>
-      <c r="AE25" s="334"/>
-      <c r="AF25" s="334"/>
-      <c r="AG25" s="334"/>
-      <c r="AH25" s="334"/>
+      <c r="AE25" s="333"/>
+      <c r="AF25" s="333"/>
+      <c r="AG25" s="333"/>
+      <c r="AH25" s="333"/>
       <c r="AJ25" s="222" t="s">
         <v>552</v>
       </c>
@@ -9795,15 +9801,15 @@
       <c r="N29" s="105" t="s">
         <v>354</v>
       </c>
-      <c r="V29" s="334" t="s">
+      <c r="V29" s="333" t="s">
         <v>212</v>
       </c>
-      <c r="W29" s="334"/>
-      <c r="X29" s="334"/>
-      <c r="Y29" s="334"/>
-      <c r="Z29" s="334"/>
-      <c r="AA29" s="334"/>
-      <c r="AB29" s="334"/>
+      <c r="W29" s="333"/>
+      <c r="X29" s="333"/>
+      <c r="Y29" s="333"/>
+      <c r="Z29" s="333"/>
+      <c r="AA29" s="333"/>
+      <c r="AB29" s="333"/>
     </row>
     <row r="30" spans="1:42">
       <c r="A30" s="105"/>
@@ -9861,15 +9867,15 @@
       </c>
       <c r="AA30" s="27"/>
       <c r="AB30" s="27"/>
-      <c r="AJ30" s="334" t="s">
+      <c r="AJ30" s="333" t="s">
         <v>776</v>
       </c>
-      <c r="AK30" s="334"/>
-      <c r="AL30" s="334"/>
-      <c r="AM30" s="334"/>
-      <c r="AN30" s="334"/>
-      <c r="AO30" s="334"/>
-      <c r="AP30" s="334"/>
+      <c r="AK30" s="333"/>
+      <c r="AL30" s="333"/>
+      <c r="AM30" s="333"/>
+      <c r="AN30" s="333"/>
+      <c r="AO30" s="333"/>
+      <c r="AP30" s="333"/>
     </row>
     <row r="31" spans="1:42">
       <c r="B31" s="22"/>
@@ -9924,9 +9930,13 @@
     <row r="32" spans="1:42">
       <c r="T32" s="22"/>
       <c r="U32" s="22"/>
-      <c r="V32" s="22"/>
+      <c r="V32" s="22" t="s">
+        <v>1350</v>
+      </c>
       <c r="W32" s="22"/>
-      <c r="X32" s="22"/>
+      <c r="X32" s="22" t="s">
+        <v>1351</v>
+      </c>
       <c r="Y32" s="22"/>
       <c r="Z32" s="22"/>
       <c r="AJ32" t="s">
@@ -9972,13 +9982,13 @@
     </row>
     <row r="37" spans="20:36">
       <c r="T37" s="207"/>
-      <c r="V37" s="334" t="s">
+      <c r="V37" s="333" t="s">
         <v>9</v>
       </c>
-      <c r="W37" s="334"/>
-      <c r="X37" s="334"/>
-      <c r="Y37" s="334"/>
-      <c r="Z37" s="334"/>
+      <c r="W37" s="333"/>
+      <c r="X37" s="333"/>
+      <c r="Y37" s="333"/>
+      <c r="Z37" s="333"/>
       <c r="AA37" s="209"/>
       <c r="AB37" s="209"/>
       <c r="AC37" s="207"/>
@@ -10007,11 +10017,11 @@
       <c r="AA38" s="210"/>
       <c r="AB38" s="210"/>
       <c r="AC38" s="207"/>
-      <c r="AD38" s="335" t="s">
+      <c r="AD38" s="338" t="s">
         <v>260</v>
       </c>
-      <c r="AE38" s="336"/>
-      <c r="AF38" s="337"/>
+      <c r="AE38" s="339"/>
+      <c r="AF38" s="340"/>
       <c r="AG38" s="207"/>
     </row>
     <row r="39" spans="20:36">
@@ -10143,15 +10153,15 @@
       <c r="AG43" s="207"/>
     </row>
     <row r="44" spans="20:36">
-      <c r="V44" s="334" t="s">
+      <c r="V44" s="333" t="s">
         <v>244</v>
       </c>
-      <c r="W44" s="334"/>
-      <c r="X44" s="334"/>
-      <c r="Y44" s="334"/>
-      <c r="Z44" s="334"/>
-      <c r="AA44" s="334"/>
-      <c r="AB44" s="334"/>
+      <c r="W44" s="333"/>
+      <c r="X44" s="333"/>
+      <c r="Y44" s="333"/>
+      <c r="Z44" s="333"/>
+      <c r="AA44" s="333"/>
+      <c r="AB44" s="333"/>
       <c r="AC44" s="207"/>
       <c r="AD44" s="3" t="s">
         <v>256</v>
@@ -10230,15 +10240,15 @@
       <c r="AG47" s="207"/>
     </row>
     <row r="48" spans="20:36">
-      <c r="V48" s="338" t="s">
+      <c r="V48" s="334" t="s">
         <v>472</v>
       </c>
-      <c r="W48" s="339"/>
-      <c r="X48" s="339"/>
-      <c r="Y48" s="339"/>
-      <c r="Z48" s="339"/>
-      <c r="AA48" s="339"/>
-      <c r="AB48" s="340"/>
+      <c r="W48" s="335"/>
+      <c r="X48" s="335"/>
+      <c r="Y48" s="335"/>
+      <c r="Z48" s="335"/>
+      <c r="AA48" s="335"/>
+      <c r="AB48" s="336"/>
       <c r="AC48" s="207"/>
       <c r="AD48" s="3" t="s">
         <v>261</v>
@@ -11074,11 +11084,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="V44:AB44"/>
-    <mergeCell ref="AD4:AH4"/>
-    <mergeCell ref="V2:Z2"/>
-    <mergeCell ref="V48:AB48"/>
-    <mergeCell ref="V37:Z37"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="R20:T20"/>
     <mergeCell ref="AJ4:AP4"/>
@@ -11087,6 +11092,11 @@
     <mergeCell ref="V29:AB29"/>
     <mergeCell ref="AD25:AH25"/>
     <mergeCell ref="AJ30:AP30"/>
+    <mergeCell ref="V44:AB44"/>
+    <mergeCell ref="AD4:AH4"/>
+    <mergeCell ref="V2:Z2"/>
+    <mergeCell ref="V48:AB48"/>
+    <mergeCell ref="V37:Z37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -12036,40 +12046,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
-      <c r="A1" s="466" t="s">
+      <c r="A1" s="449" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="466"/>
-      <c r="C1" s="466"/>
-      <c r="D1" s="466"/>
-      <c r="E1" s="466"/>
-      <c r="F1" s="466"/>
-      <c r="G1" s="466"/>
-      <c r="H1" s="466"/>
+      <c r="B1" s="449"/>
+      <c r="C1" s="449"/>
+      <c r="D1" s="449"/>
+      <c r="E1" s="449"/>
+      <c r="F1" s="449"/>
+      <c r="G1" s="449"/>
+      <c r="H1" s="449"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A2" s="467"/>
-      <c r="B2" s="467"/>
-      <c r="C2" s="467"/>
-      <c r="D2" s="467"/>
-      <c r="E2" s="467"/>
-      <c r="F2" s="467"/>
-      <c r="G2" s="467"/>
-      <c r="H2" s="467"/>
+      <c r="A2" s="450"/>
+      <c r="B2" s="450"/>
+      <c r="C2" s="450"/>
+      <c r="D2" s="450"/>
+      <c r="E2" s="450"/>
+      <c r="F2" s="450"/>
+      <c r="G2" s="450"/>
+      <c r="H2" s="450"/>
     </row>
     <row r="3" spans="1:8" ht="24" thickBot="1">
-      <c r="A3" s="468" t="s">
+      <c r="A3" s="451" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="469"/>
-      <c r="C3" s="470"/>
-      <c r="D3" s="471"/>
-      <c r="E3" s="468" t="s">
+      <c r="B3" s="452"/>
+      <c r="C3" s="453"/>
+      <c r="D3" s="454"/>
+      <c r="E3" s="451" t="s">
         <v>228</v>
       </c>
-      <c r="F3" s="469"/>
-      <c r="G3" s="470"/>
-      <c r="H3" s="471"/>
+      <c r="F3" s="452"/>
+      <c r="G3" s="453"/>
+      <c r="H3" s="454"/>
     </row>
     <row r="4" spans="1:8" ht="18">
       <c r="A4" s="29">
@@ -12362,18 +12372,18 @@
       <c r="H24" s="57"/>
     </row>
     <row r="25" spans="1:8" ht="24" thickBot="1">
-      <c r="A25" s="468" t="s">
+      <c r="A25" s="451" t="s">
         <v>289</v>
       </c>
-      <c r="B25" s="469"/>
-      <c r="C25" s="470"/>
-      <c r="D25" s="471"/>
-      <c r="E25" s="468" t="s">
+      <c r="B25" s="452"/>
+      <c r="C25" s="453"/>
+      <c r="D25" s="454"/>
+      <c r="E25" s="451" t="s">
         <v>290</v>
       </c>
-      <c r="F25" s="469"/>
-      <c r="G25" s="470"/>
-      <c r="H25" s="471"/>
+      <c r="F25" s="452"/>
+      <c r="G25" s="453"/>
+      <c r="H25" s="454"/>
     </row>
     <row r="26" spans="1:8" ht="18.75" thickBot="1">
       <c r="A26" s="33" t="s">
@@ -12385,23 +12395,23 @@
       <c r="E26" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="F26" s="463"/>
-      <c r="G26" s="464"/>
-      <c r="H26" s="465"/>
+      <c r="F26" s="458"/>
+      <c r="G26" s="459"/>
+      <c r="H26" s="460"/>
     </row>
     <row r="27" spans="1:8" ht="18.75" thickBot="1">
       <c r="A27" s="41" t="s">
         <v>293</v>
       </c>
-      <c r="B27" s="458"/>
-      <c r="C27" s="459"/>
-      <c r="D27" s="461"/>
+      <c r="B27" s="461"/>
+      <c r="C27" s="462"/>
+      <c r="D27" s="463"/>
       <c r="E27" s="33" t="s">
         <v>294</v>
       </c>
       <c r="F27" s="455"/>
       <c r="G27" s="456"/>
-      <c r="H27" s="462"/>
+      <c r="H27" s="464"/>
     </row>
     <row r="28" spans="1:8" ht="18.75" thickBot="1">
       <c r="A28" s="33" t="s">
@@ -12413,23 +12423,23 @@
       <c r="E28" s="41" t="s">
         <v>296</v>
       </c>
-      <c r="F28" s="458"/>
-      <c r="G28" s="459"/>
-      <c r="H28" s="460"/>
+      <c r="F28" s="461"/>
+      <c r="G28" s="462"/>
+      <c r="H28" s="465"/>
     </row>
     <row r="29" spans="1:8" ht="18.75" thickBot="1">
       <c r="A29" s="41" t="s">
         <v>297</v>
       </c>
-      <c r="B29" s="458"/>
-      <c r="C29" s="459"/>
-      <c r="D29" s="461"/>
+      <c r="B29" s="461"/>
+      <c r="C29" s="462"/>
+      <c r="D29" s="463"/>
       <c r="E29" s="33" t="s">
         <v>298</v>
       </c>
       <c r="F29" s="455"/>
       <c r="G29" s="456"/>
-      <c r="H29" s="462"/>
+      <c r="H29" s="464"/>
     </row>
     <row r="30" spans="1:8" ht="18.75" thickBot="1">
       <c r="A30" s="33" t="s">
@@ -12441,23 +12451,23 @@
       <c r="E30" s="41" t="s">
         <v>300</v>
       </c>
-      <c r="F30" s="458"/>
-      <c r="G30" s="459"/>
-      <c r="H30" s="460"/>
+      <c r="F30" s="461"/>
+      <c r="G30" s="462"/>
+      <c r="H30" s="465"/>
     </row>
     <row r="31" spans="1:8" ht="18.75" thickBot="1">
       <c r="A31" s="41" t="s">
         <v>301</v>
       </c>
-      <c r="B31" s="458"/>
-      <c r="C31" s="459"/>
-      <c r="D31" s="461"/>
+      <c r="B31" s="461"/>
+      <c r="C31" s="462"/>
+      <c r="D31" s="463"/>
       <c r="E31" s="33" t="s">
         <v>302</v>
       </c>
       <c r="F31" s="455"/>
       <c r="G31" s="456"/>
-      <c r="H31" s="462"/>
+      <c r="H31" s="464"/>
     </row>
     <row r="32" spans="1:8" ht="18.75" thickBot="1">
       <c r="A32" s="33" t="s">
@@ -12467,9 +12477,9 @@
       <c r="C32" s="456"/>
       <c r="D32" s="457"/>
       <c r="E32" s="41"/>
-      <c r="F32" s="458"/>
-      <c r="G32" s="459"/>
-      <c r="H32" s="460" t="s">
+      <c r="F32" s="461"/>
+      <c r="G32" s="462"/>
+      <c r="H32" s="465" t="s">
         <v>242</v>
       </c>
     </row>
@@ -12477,13 +12487,13 @@
       <c r="A33" s="41" t="s">
         <v>304</v>
       </c>
-      <c r="B33" s="458"/>
-      <c r="C33" s="459"/>
-      <c r="D33" s="461"/>
+      <c r="B33" s="461"/>
+      <c r="C33" s="462"/>
+      <c r="D33" s="463"/>
       <c r="E33" s="33"/>
       <c r="F33" s="455"/>
       <c r="G33" s="456"/>
-      <c r="H33" s="462" t="s">
+      <c r="H33" s="464" t="s">
         <v>284</v>
       </c>
     </row>
@@ -12495,9 +12505,9 @@
       <c r="C34" s="456"/>
       <c r="D34" s="457"/>
       <c r="E34" s="41"/>
-      <c r="F34" s="458"/>
-      <c r="G34" s="459"/>
-      <c r="H34" s="460" t="s">
+      <c r="F34" s="461"/>
+      <c r="G34" s="462"/>
+      <c r="H34" s="465" t="s">
         <v>285</v>
       </c>
     </row>
@@ -12505,13 +12515,13 @@
       <c r="A35" s="41" t="s">
         <v>306</v>
       </c>
-      <c r="B35" s="458"/>
-      <c r="C35" s="459"/>
-      <c r="D35" s="461"/>
+      <c r="B35" s="461"/>
+      <c r="C35" s="462"/>
+      <c r="D35" s="463"/>
       <c r="E35" s="33"/>
       <c r="F35" s="455"/>
       <c r="G35" s="456"/>
-      <c r="H35" s="462" t="s">
+      <c r="H35" s="464" t="s">
         <v>286</v>
       </c>
     </row>
@@ -12523,9 +12533,9 @@
       <c r="C36" s="456"/>
       <c r="D36" s="457"/>
       <c r="E36" s="41"/>
-      <c r="F36" s="458"/>
-      <c r="G36" s="459"/>
-      <c r="H36" s="460" t="s">
+      <c r="F36" s="461"/>
+      <c r="G36" s="462"/>
+      <c r="H36" s="465" t="s">
         <v>287</v>
       </c>
     </row>
@@ -12533,13 +12543,13 @@
       <c r="A37" s="41" t="s">
         <v>308</v>
       </c>
-      <c r="B37" s="458"/>
-      <c r="C37" s="459"/>
-      <c r="D37" s="461"/>
+      <c r="B37" s="461"/>
+      <c r="C37" s="462"/>
+      <c r="D37" s="463"/>
       <c r="E37" s="33"/>
       <c r="F37" s="455"/>
       <c r="G37" s="456"/>
-      <c r="H37" s="462" t="s">
+      <c r="H37" s="464" t="s">
         <v>288</v>
       </c>
     </row>
@@ -12551,9 +12561,9 @@
       <c r="C38" s="456"/>
       <c r="D38" s="457"/>
       <c r="E38" s="41"/>
-      <c r="F38" s="458"/>
-      <c r="G38" s="459"/>
-      <c r="H38" s="460" t="s">
+      <c r="F38" s="461"/>
+      <c r="G38" s="462"/>
+      <c r="H38" s="465" t="s">
         <v>241</v>
       </c>
     </row>
@@ -12561,13 +12571,13 @@
       <c r="A39" s="41" t="s">
         <v>310</v>
       </c>
-      <c r="B39" s="458"/>
-      <c r="C39" s="459"/>
-      <c r="D39" s="461"/>
+      <c r="B39" s="461"/>
+      <c r="C39" s="462"/>
+      <c r="D39" s="463"/>
       <c r="E39" s="33"/>
       <c r="F39" s="455"/>
       <c r="G39" s="456"/>
-      <c r="H39" s="462" t="s">
+      <c r="H39" s="464" t="s">
         <v>242</v>
       </c>
     </row>
@@ -12579,53 +12589,24 @@
       <c r="C40" s="456"/>
       <c r="D40" s="457"/>
       <c r="E40" s="41"/>
-      <c r="F40" s="458"/>
-      <c r="G40" s="459"/>
-      <c r="H40" s="460"/>
+      <c r="F40" s="461"/>
+      <c r="G40" s="462"/>
+      <c r="H40" s="465"/>
     </row>
     <row r="41" spans="1:8" ht="18.75" thickBot="1">
       <c r="A41" s="53" t="s">
         <v>312</v>
       </c>
-      <c r="B41" s="449"/>
-      <c r="C41" s="450"/>
-      <c r="D41" s="451"/>
+      <c r="B41" s="466"/>
+      <c r="C41" s="467"/>
+      <c r="D41" s="468"/>
       <c r="E41" s="58"/>
-      <c r="F41" s="452"/>
-      <c r="G41" s="453"/>
-      <c r="H41" s="454"/>
+      <c r="F41" s="469"/>
+      <c r="G41" s="470"/>
+      <c r="H41" s="471"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="F37:H37"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="F41:H41"/>
     <mergeCell ref="B38:D38"/>
@@ -12634,6 +12615,35 @@
     <mergeCell ref="F39:H39"/>
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="F40:H40"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="F37:H37"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="E25:H25"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -12790,10 +12800,10 @@
       <c r="B8" s="475" t="s">
         <v>274</v>
       </c>
-      <c r="C8" s="334"/>
-      <c r="D8" s="334"/>
-      <c r="E8" s="334"/>
-      <c r="F8" s="334"/>
+      <c r="C8" s="333"/>
+      <c r="D8" s="333"/>
+      <c r="E8" s="333"/>
+      <c r="F8" s="333"/>
       <c r="G8" s="476"/>
       <c r="H8" s="207"/>
     </row>
@@ -12912,10 +12922,10 @@
       <c r="B14" s="475" t="s">
         <v>776</v>
       </c>
-      <c r="C14" s="334"/>
-      <c r="D14" s="334"/>
-      <c r="E14" s="334"/>
-      <c r="F14" s="334"/>
+      <c r="C14" s="333"/>
+      <c r="D14" s="333"/>
+      <c r="E14" s="333"/>
+      <c r="F14" s="333"/>
       <c r="G14" s="476"/>
       <c r="H14" s="207"/>
     </row>
@@ -13033,55 +13043,55 @@
       </c>
     </row>
     <row r="2" spans="2:42">
-      <c r="B2" s="334" t="s">
+      <c r="B2" s="333" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="334"/>
-      <c r="D2" s="334"/>
-      <c r="E2" s="334"/>
-      <c r="F2" s="334"/>
-      <c r="H2" s="334" t="s">
+      <c r="C2" s="333"/>
+      <c r="D2" s="333"/>
+      <c r="E2" s="333"/>
+      <c r="F2" s="333"/>
+      <c r="H2" s="333" t="s">
         <v>959</v>
       </c>
-      <c r="I2" s="334"/>
-      <c r="J2" s="334"/>
-      <c r="K2" s="334"/>
-      <c r="L2" s="334"/>
-      <c r="N2" s="334" t="s">
+      <c r="I2" s="333"/>
+      <c r="J2" s="333"/>
+      <c r="K2" s="333"/>
+      <c r="L2" s="333"/>
+      <c r="N2" s="333" t="s">
         <v>958</v>
       </c>
-      <c r="O2" s="334"/>
-      <c r="P2" s="334"/>
-      <c r="Q2" s="334"/>
-      <c r="R2" s="334"/>
-      <c r="T2" s="334" t="s">
+      <c r="O2" s="333"/>
+      <c r="P2" s="333"/>
+      <c r="Q2" s="333"/>
+      <c r="R2" s="333"/>
+      <c r="T2" s="333" t="s">
         <v>236</v>
       </c>
-      <c r="U2" s="334"/>
-      <c r="V2" s="334"/>
-      <c r="W2" s="334"/>
-      <c r="X2" s="334"/>
-      <c r="Z2" s="334" t="s">
+      <c r="U2" s="333"/>
+      <c r="V2" s="333"/>
+      <c r="W2" s="333"/>
+      <c r="X2" s="333"/>
+      <c r="Z2" s="333" t="s">
         <v>246</v>
       </c>
-      <c r="AA2" s="334"/>
-      <c r="AB2" s="334"/>
-      <c r="AC2" s="334"/>
-      <c r="AD2" s="334"/>
-      <c r="AF2" s="334" t="s">
+      <c r="AA2" s="333"/>
+      <c r="AB2" s="333"/>
+      <c r="AC2" s="333"/>
+      <c r="AD2" s="333"/>
+      <c r="AF2" s="333" t="s">
         <v>317</v>
       </c>
-      <c r="AG2" s="334"/>
-      <c r="AH2" s="334"/>
-      <c r="AI2" s="334"/>
-      <c r="AJ2" s="334"/>
-      <c r="AL2" s="334" t="s">
+      <c r="AG2" s="333"/>
+      <c r="AH2" s="333"/>
+      <c r="AI2" s="333"/>
+      <c r="AJ2" s="333"/>
+      <c r="AL2" s="333" t="s">
         <v>490</v>
       </c>
-      <c r="AM2" s="334"/>
-      <c r="AN2" s="334"/>
-      <c r="AO2" s="334"/>
-      <c r="AP2" s="334"/>
+      <c r="AM2" s="333"/>
+      <c r="AN2" s="333"/>
+      <c r="AO2" s="333"/>
+      <c r="AP2" s="333"/>
     </row>
     <row r="3" spans="2:42">
       <c r="B3" s="99" t="s">
@@ -14747,20 +14757,20 @@
       </c>
     </row>
     <row r="41" spans="2:28">
-      <c r="B41" s="334" t="s">
+      <c r="B41" s="333" t="s">
         <v>643</v>
       </c>
-      <c r="C41" s="334"/>
-      <c r="D41" s="334"/>
-      <c r="E41" s="334"/>
-      <c r="F41" s="334"/>
-      <c r="H41" s="334" t="s">
+      <c r="C41" s="333"/>
+      <c r="D41" s="333"/>
+      <c r="E41" s="333"/>
+      <c r="F41" s="333"/>
+      <c r="H41" s="333" t="s">
         <v>695</v>
       </c>
-      <c r="I41" s="334"/>
-      <c r="J41" s="334"/>
-      <c r="K41" s="334"/>
-      <c r="L41" s="334"/>
+      <c r="I41" s="333"/>
+      <c r="J41" s="333"/>
+      <c r="K41" s="333"/>
+      <c r="L41" s="333"/>
     </row>
     <row r="42" spans="2:28">
       <c r="B42" s="99" t="s">
@@ -15354,39 +15364,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27" customHeight="1" thickBot="1">
-      <c r="A1" s="350" t="s">
+      <c r="A1" s="352" t="s">
         <v>1192</v>
       </c>
-      <c r="B1" s="351"/>
-      <c r="C1" s="351"/>
-      <c r="D1" s="351"/>
-      <c r="E1" s="351"/>
-      <c r="F1" s="351"/>
-      <c r="G1" s="351"/>
-      <c r="H1" s="351"/>
-      <c r="I1" s="351"/>
-      <c r="J1" s="351"/>
-      <c r="K1" s="351"/>
-      <c r="L1" s="352"/>
+      <c r="B1" s="353"/>
+      <c r="C1" s="353"/>
+      <c r="D1" s="353"/>
+      <c r="E1" s="353"/>
+      <c r="F1" s="353"/>
+      <c r="G1" s="353"/>
+      <c r="H1" s="353"/>
+      <c r="I1" s="353"/>
+      <c r="J1" s="353"/>
+      <c r="K1" s="353"/>
+      <c r="L1" s="354"/>
     </row>
     <row r="2" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A2" s="347" t="s">
+      <c r="A2" s="349" t="s">
         <v>1293</v>
       </c>
-      <c r="B2" s="348"/>
-      <c r="C2" s="349"/>
+      <c r="B2" s="350"/>
+      <c r="C2" s="351"/>
       <c r="D2" s="325"/>
-      <c r="E2" s="347" t="s">
+      <c r="E2" s="349" t="s">
         <v>1294</v>
       </c>
-      <c r="F2" s="348"/>
-      <c r="G2" s="349"/>
+      <c r="F2" s="350"/>
+      <c r="G2" s="351"/>
       <c r="H2" s="325"/>
-      <c r="I2" s="347" t="s">
+      <c r="I2" s="349" t="s">
         <v>958</v>
       </c>
-      <c r="J2" s="348"/>
-      <c r="K2" s="349"/>
+      <c r="J2" s="350"/>
+      <c r="K2" s="351"/>
       <c r="L2" s="117"/>
     </row>
     <row r="3" spans="1:12" ht="19.5" thickBot="1">
@@ -15422,7 +15432,7 @@
       <c r="L3" s="117"/>
     </row>
     <row r="4" spans="1:12" ht="18.75">
-      <c r="A4" s="341" t="s">
+      <c r="A4" s="342" t="s">
         <v>325</v>
       </c>
       <c r="B4" s="123" t="s">
@@ -15432,7 +15442,7 @@
         <v>650</v>
       </c>
       <c r="D4" s="248"/>
-      <c r="E4" s="344" t="s">
+      <c r="E4" s="346" t="s">
         <v>1295</v>
       </c>
       <c r="F4" s="123" t="s">
@@ -15442,7 +15452,7 @@
         <v>932</v>
       </c>
       <c r="H4" s="246"/>
-      <c r="I4" s="344" t="s">
+      <c r="I4" s="346" t="s">
         <v>1295</v>
       </c>
       <c r="J4" s="123" t="s">
@@ -15454,7 +15464,7 @@
       <c r="L4" s="117"/>
     </row>
     <row r="5" spans="1:12" ht="18.75">
-      <c r="A5" s="342"/>
+      <c r="A5" s="343"/>
       <c r="B5" s="122" t="s">
         <v>322</v>
       </c>
@@ -15462,7 +15472,7 @@
         <v>651</v>
       </c>
       <c r="D5" s="248"/>
-      <c r="E5" s="345"/>
+      <c r="E5" s="347"/>
       <c r="F5" s="122" t="s">
         <v>906</v>
       </c>
@@ -15470,7 +15480,7 @@
         <v>933</v>
       </c>
       <c r="H5" s="246"/>
-      <c r="I5" s="345"/>
+      <c r="I5" s="347"/>
       <c r="J5" s="122" t="s">
         <v>996</v>
       </c>
@@ -15480,7 +15490,7 @@
       <c r="L5" s="117"/>
     </row>
     <row r="6" spans="1:12" ht="18.75">
-      <c r="A6" s="342"/>
+      <c r="A6" s="343"/>
       <c r="B6" s="122" t="s">
         <v>323</v>
       </c>
@@ -15488,7 +15498,7 @@
         <v>652</v>
       </c>
       <c r="D6" s="248"/>
-      <c r="E6" s="345"/>
+      <c r="E6" s="347"/>
       <c r="F6" s="122" t="s">
         <v>907</v>
       </c>
@@ -15496,7 +15506,7 @@
         <v>934</v>
       </c>
       <c r="H6" s="246"/>
-      <c r="I6" s="345"/>
+      <c r="I6" s="347"/>
       <c r="J6" s="122" t="s">
         <v>997</v>
       </c>
@@ -15506,7 +15516,7 @@
       <c r="L6" s="117"/>
     </row>
     <row r="7" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A7" s="343"/>
+      <c r="A7" s="344"/>
       <c r="B7" s="126" t="s">
         <v>324</v>
       </c>
@@ -15514,7 +15524,7 @@
         <v>653</v>
       </c>
       <c r="D7" s="248"/>
-      <c r="E7" s="346"/>
+      <c r="E7" s="348"/>
       <c r="F7" s="126" t="s">
         <v>908</v>
       </c>
@@ -15522,7 +15532,7 @@
         <v>935</v>
       </c>
       <c r="H7" s="246"/>
-      <c r="I7" s="346"/>
+      <c r="I7" s="348"/>
       <c r="J7" s="126" t="s">
         <v>998</v>
       </c>
@@ -15532,7 +15542,7 @@
       <c r="L7" s="117"/>
     </row>
     <row r="8" spans="1:12" ht="18.75">
-      <c r="A8" s="341" t="s">
+      <c r="A8" s="342" t="s">
         <v>613</v>
       </c>
       <c r="B8" s="123" t="s">
@@ -15542,7 +15552,7 @@
         <v>654</v>
       </c>
       <c r="D8" s="248"/>
-      <c r="E8" s="344" t="s">
+      <c r="E8" s="346" t="s">
         <v>962</v>
       </c>
       <c r="F8" s="123" t="s">
@@ -15552,7 +15562,7 @@
         <v>936</v>
       </c>
       <c r="H8" s="246"/>
-      <c r="I8" s="344" t="s">
+      <c r="I8" s="346" t="s">
         <v>962</v>
       </c>
       <c r="J8" s="123" t="s">
@@ -15564,7 +15574,7 @@
       <c r="L8" s="117"/>
     </row>
     <row r="9" spans="1:12" ht="18.75">
-      <c r="A9" s="342"/>
+      <c r="A9" s="343"/>
       <c r="B9" s="122" t="s">
         <v>604</v>
       </c>
@@ -15572,7 +15582,7 @@
         <v>655</v>
       </c>
       <c r="D9" s="248"/>
-      <c r="E9" s="345"/>
+      <c r="E9" s="347"/>
       <c r="F9" s="122" t="s">
         <v>910</v>
       </c>
@@ -15580,7 +15590,7 @@
         <v>937</v>
       </c>
       <c r="H9" s="246"/>
-      <c r="I9" s="345"/>
+      <c r="I9" s="347"/>
       <c r="J9" s="122" t="s">
         <v>999</v>
       </c>
@@ -15590,7 +15600,7 @@
       <c r="L9" s="117"/>
     </row>
     <row r="10" spans="1:12" ht="18.75">
-      <c r="A10" s="342"/>
+      <c r="A10" s="343"/>
       <c r="B10" s="122" t="s">
         <v>605</v>
       </c>
@@ -15598,7 +15608,7 @@
         <v>656</v>
       </c>
       <c r="D10" s="248"/>
-      <c r="E10" s="345"/>
+      <c r="E10" s="347"/>
       <c r="F10" s="122" t="s">
         <v>912</v>
       </c>
@@ -15606,7 +15616,7 @@
         <v>938</v>
       </c>
       <c r="H10" s="246"/>
-      <c r="I10" s="345"/>
+      <c r="I10" s="347"/>
       <c r="J10" s="122" t="s">
         <v>1000</v>
       </c>
@@ -15616,7 +15626,7 @@
       <c r="L10" s="117"/>
     </row>
     <row r="11" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A11" s="343"/>
+      <c r="A11" s="344"/>
       <c r="B11" s="126" t="s">
         <v>606</v>
       </c>
@@ -15624,7 +15634,7 @@
         <v>657</v>
       </c>
       <c r="D11" s="248"/>
-      <c r="E11" s="346"/>
+      <c r="E11" s="348"/>
       <c r="F11" s="126" t="s">
         <v>913</v>
       </c>
@@ -15632,7 +15642,7 @@
         <v>939</v>
       </c>
       <c r="H11" s="246"/>
-      <c r="I11" s="346"/>
+      <c r="I11" s="348"/>
       <c r="J11" s="126" t="s">
         <v>1001</v>
       </c>
@@ -15642,7 +15652,7 @@
       <c r="L11" s="117"/>
     </row>
     <row r="12" spans="1:12" ht="18.75">
-      <c r="A12" s="341" t="s">
+      <c r="A12" s="342" t="s">
         <v>611</v>
       </c>
       <c r="B12" s="123" t="s">
@@ -15652,7 +15662,7 @@
         <v>658</v>
       </c>
       <c r="D12" s="248"/>
-      <c r="E12" s="344" t="s">
+      <c r="E12" s="346" t="s">
         <v>1296</v>
       </c>
       <c r="F12" s="123" t="s">
@@ -15662,7 +15672,7 @@
         <v>940</v>
       </c>
       <c r="H12" s="246"/>
-      <c r="I12" s="344" t="s">
+      <c r="I12" s="346" t="s">
         <v>1296</v>
       </c>
       <c r="J12" s="123" t="s">
@@ -15674,7 +15684,7 @@
       <c r="L12" s="117"/>
     </row>
     <row r="13" spans="1:12" ht="18.75">
-      <c r="A13" s="342"/>
+      <c r="A13" s="343"/>
       <c r="B13" s="122" t="s">
         <v>608</v>
       </c>
@@ -15682,7 +15692,7 @@
         <v>659</v>
       </c>
       <c r="D13" s="248"/>
-      <c r="E13" s="345"/>
+      <c r="E13" s="347"/>
       <c r="F13" s="122" t="s">
         <v>915</v>
       </c>
@@ -15690,7 +15700,7 @@
         <v>941</v>
       </c>
       <c r="H13" s="246"/>
-      <c r="I13" s="345"/>
+      <c r="I13" s="347"/>
       <c r="J13" s="122" t="s">
         <v>1003</v>
       </c>
@@ -15700,7 +15710,7 @@
       <c r="L13" s="117"/>
     </row>
     <row r="14" spans="1:12" ht="18.75">
-      <c r="A14" s="342"/>
+      <c r="A14" s="343"/>
       <c r="B14" s="122" t="s">
         <v>609</v>
       </c>
@@ -15708,7 +15718,7 @@
         <v>660</v>
       </c>
       <c r="D14" s="248"/>
-      <c r="E14" s="345"/>
+      <c r="E14" s="347"/>
       <c r="F14" s="122" t="s">
         <v>916</v>
       </c>
@@ -15716,7 +15726,7 @@
         <v>942</v>
       </c>
       <c r="H14" s="246"/>
-      <c r="I14" s="345"/>
+      <c r="I14" s="347"/>
       <c r="J14" s="122" t="s">
         <v>1004</v>
       </c>
@@ -15726,7 +15736,7 @@
       <c r="L14" s="117"/>
     </row>
     <row r="15" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A15" s="343"/>
+      <c r="A15" s="344"/>
       <c r="B15" s="126" t="s">
         <v>610</v>
       </c>
@@ -15734,7 +15744,7 @@
         <v>661</v>
       </c>
       <c r="D15" s="248"/>
-      <c r="E15" s="346"/>
+      <c r="E15" s="348"/>
       <c r="F15" s="126" t="s">
         <v>917</v>
       </c>
@@ -15742,7 +15752,7 @@
         <v>943</v>
       </c>
       <c r="H15" s="246"/>
-      <c r="I15" s="346"/>
+      <c r="I15" s="348"/>
       <c r="J15" s="126" t="s">
         <v>1005</v>
       </c>
@@ -15752,7 +15762,7 @@
       <c r="L15" s="117"/>
     </row>
     <row r="16" spans="1:12" ht="18.75">
-      <c r="A16" s="341" t="s">
+      <c r="A16" s="342" t="s">
         <v>1258</v>
       </c>
       <c r="B16" s="123" t="s">
@@ -15762,7 +15772,7 @@
         <v>662</v>
       </c>
       <c r="D16" s="248"/>
-      <c r="E16" s="344" t="s">
+      <c r="E16" s="346" t="s">
         <v>1297</v>
       </c>
       <c r="F16" s="123" t="s">
@@ -15772,7 +15782,7 @@
         <v>944</v>
       </c>
       <c r="H16" s="246"/>
-      <c r="I16" s="344" t="s">
+      <c r="I16" s="346" t="s">
         <v>1297</v>
       </c>
       <c r="J16" s="123" t="s">
@@ -15784,7 +15794,7 @@
       <c r="L16" s="117"/>
     </row>
     <row r="17" spans="1:12" ht="18.75">
-      <c r="A17" s="342"/>
+      <c r="A17" s="343"/>
       <c r="B17" s="122" t="s">
         <v>1260</v>
       </c>
@@ -15792,7 +15802,7 @@
         <v>663</v>
       </c>
       <c r="D17" s="248"/>
-      <c r="E17" s="345"/>
+      <c r="E17" s="347"/>
       <c r="F17" s="122" t="s">
         <v>919</v>
       </c>
@@ -15800,7 +15810,7 @@
         <v>945</v>
       </c>
       <c r="H17" s="246"/>
-      <c r="I17" s="345"/>
+      <c r="I17" s="347"/>
       <c r="J17" s="122" t="s">
         <v>1007</v>
       </c>
@@ -15810,7 +15820,7 @@
       <c r="L17" s="117"/>
     </row>
     <row r="18" spans="1:12" ht="18.75">
-      <c r="A18" s="342"/>
+      <c r="A18" s="343"/>
       <c r="B18" s="122" t="s">
         <v>1261</v>
       </c>
@@ -15818,7 +15828,7 @@
         <v>664</v>
       </c>
       <c r="D18" s="248"/>
-      <c r="E18" s="345"/>
+      <c r="E18" s="347"/>
       <c r="F18" s="122" t="s">
         <v>920</v>
       </c>
@@ -15826,7 +15836,7 @@
         <v>946</v>
       </c>
       <c r="H18" s="246"/>
-      <c r="I18" s="345"/>
+      <c r="I18" s="347"/>
       <c r="J18" s="122" t="s">
         <v>1008</v>
       </c>
@@ -15836,7 +15846,7 @@
       <c r="L18" s="117"/>
     </row>
     <row r="19" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A19" s="343"/>
+      <c r="A19" s="344"/>
       <c r="B19" s="126" t="s">
         <v>1262</v>
       </c>
@@ -15844,7 +15854,7 @@
         <v>665</v>
       </c>
       <c r="D19" s="248"/>
-      <c r="E19" s="346"/>
+      <c r="E19" s="348"/>
       <c r="F19" s="126" t="s">
         <v>921</v>
       </c>
@@ -15852,7 +15862,7 @@
         <v>947</v>
       </c>
       <c r="H19" s="246"/>
-      <c r="I19" s="346"/>
+      <c r="I19" s="348"/>
       <c r="J19" s="126" t="s">
         <v>1009</v>
       </c>
@@ -15862,7 +15872,7 @@
       <c r="L19" s="117"/>
     </row>
     <row r="20" spans="1:12" ht="18.75">
-      <c r="A20" s="341" t="s">
+      <c r="A20" s="342" t="s">
         <v>1263</v>
       </c>
       <c r="B20" s="123" t="s">
@@ -15872,7 +15882,7 @@
         <v>1268</v>
       </c>
       <c r="D20" s="246"/>
-      <c r="E20" s="344" t="s">
+      <c r="E20" s="346" t="s">
         <v>1298</v>
       </c>
       <c r="F20" s="123" t="s">
@@ -15882,7 +15892,7 @@
         <v>948</v>
       </c>
       <c r="H20" s="246"/>
-      <c r="I20" s="344" t="s">
+      <c r="I20" s="346" t="s">
         <v>1298</v>
       </c>
       <c r="J20" s="123" t="s">
@@ -15894,7 +15904,7 @@
       <c r="L20" s="117"/>
     </row>
     <row r="21" spans="1:12" ht="18.75">
-      <c r="A21" s="342"/>
+      <c r="A21" s="343"/>
       <c r="B21" s="122" t="s">
         <v>1265</v>
       </c>
@@ -15902,7 +15912,7 @@
         <v>1269</v>
       </c>
       <c r="D21" s="246"/>
-      <c r="E21" s="345"/>
+      <c r="E21" s="347"/>
       <c r="F21" s="122" t="s">
         <v>923</v>
       </c>
@@ -15910,7 +15920,7 @@
         <v>949</v>
       </c>
       <c r="H21" s="246"/>
-      <c r="I21" s="345"/>
+      <c r="I21" s="347"/>
       <c r="J21" s="122" t="s">
         <v>1011</v>
       </c>
@@ -15920,7 +15930,7 @@
       <c r="L21" s="117"/>
     </row>
     <row r="22" spans="1:12" ht="18.75">
-      <c r="A22" s="342"/>
+      <c r="A22" s="343"/>
       <c r="B22" s="122" t="s">
         <v>1266</v>
       </c>
@@ -15928,7 +15938,7 @@
         <v>1270</v>
       </c>
       <c r="D22" s="246"/>
-      <c r="E22" s="345"/>
+      <c r="E22" s="347"/>
       <c r="F22" s="122" t="s">
         <v>924</v>
       </c>
@@ -15936,7 +15946,7 @@
         <v>950</v>
       </c>
       <c r="H22" s="246"/>
-      <c r="I22" s="345"/>
+      <c r="I22" s="347"/>
       <c r="J22" s="122" t="s">
         <v>1012</v>
       </c>
@@ -15946,7 +15956,7 @@
       <c r="L22" s="117"/>
     </row>
     <row r="23" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A23" s="343"/>
+      <c r="A23" s="344"/>
       <c r="B23" s="126" t="s">
         <v>1267</v>
       </c>
@@ -15954,7 +15964,7 @@
         <v>1271</v>
       </c>
       <c r="D23" s="246"/>
-      <c r="E23" s="346"/>
+      <c r="E23" s="348"/>
       <c r="F23" s="126" t="s">
         <v>925</v>
       </c>
@@ -15962,7 +15972,7 @@
         <v>951</v>
       </c>
       <c r="H23" s="246"/>
-      <c r="I23" s="346"/>
+      <c r="I23" s="348"/>
       <c r="J23" s="126" t="s">
         <v>1013</v>
       </c>
@@ -15972,7 +15982,7 @@
       <c r="L23" s="117"/>
     </row>
     <row r="24" spans="1:12" ht="18.75">
-      <c r="A24" s="341" t="s">
+      <c r="A24" s="342" t="s">
         <v>1281</v>
       </c>
       <c r="B24" s="123" t="s">
@@ -15982,7 +15992,7 @@
         <v>1272</v>
       </c>
       <c r="D24" s="246"/>
-      <c r="E24" s="344" t="s">
+      <c r="E24" s="346" t="s">
         <v>1299</v>
       </c>
       <c r="F24" s="123" t="s">
@@ -15992,7 +16002,7 @@
         <v>952</v>
       </c>
       <c r="H24" s="246"/>
-      <c r="I24" s="344" t="s">
+      <c r="I24" s="346" t="s">
         <v>1299</v>
       </c>
       <c r="J24" s="123" t="s">
@@ -16004,7 +16014,7 @@
       <c r="L24" s="117"/>
     </row>
     <row r="25" spans="1:12" ht="18.75">
-      <c r="A25" s="342"/>
+      <c r="A25" s="343"/>
       <c r="B25" s="122" t="s">
         <v>1283</v>
       </c>
@@ -16012,7 +16022,7 @@
         <v>1273</v>
       </c>
       <c r="D25" s="246"/>
-      <c r="E25" s="345"/>
+      <c r="E25" s="347"/>
       <c r="F25" s="122" t="s">
         <v>927</v>
       </c>
@@ -16020,7 +16030,7 @@
         <v>953</v>
       </c>
       <c r="H25" s="246"/>
-      <c r="I25" s="345"/>
+      <c r="I25" s="347"/>
       <c r="J25" s="122" t="s">
         <v>1015</v>
       </c>
@@ -16030,7 +16040,7 @@
       <c r="L25" s="117"/>
     </row>
     <row r="26" spans="1:12" ht="18.75">
-      <c r="A26" s="342"/>
+      <c r="A26" s="343"/>
       <c r="B26" s="122" t="s">
         <v>1284</v>
       </c>
@@ -16038,7 +16048,7 @@
         <v>1274</v>
       </c>
       <c r="D26" s="246"/>
-      <c r="E26" s="345"/>
+      <c r="E26" s="347"/>
       <c r="F26" s="122" t="s">
         <v>928</v>
       </c>
@@ -16046,7 +16056,7 @@
         <v>954</v>
       </c>
       <c r="H26" s="246"/>
-      <c r="I26" s="345"/>
+      <c r="I26" s="347"/>
       <c r="J26" s="122" t="s">
         <v>1016</v>
       </c>
@@ -16056,7 +16066,7 @@
       <c r="L26" s="117"/>
     </row>
     <row r="27" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A27" s="343"/>
+      <c r="A27" s="344"/>
       <c r="B27" s="126" t="s">
         <v>1285</v>
       </c>
@@ -16064,7 +16074,7 @@
         <v>1275</v>
       </c>
       <c r="D27" s="246"/>
-      <c r="E27" s="346"/>
+      <c r="E27" s="348"/>
       <c r="F27" s="126" t="s">
         <v>929</v>
       </c>
@@ -16072,7 +16082,7 @@
         <v>955</v>
       </c>
       <c r="H27" s="246"/>
-      <c r="I27" s="346"/>
+      <c r="I27" s="348"/>
       <c r="J27" s="126" t="s">
         <v>1017</v>
       </c>
@@ -16082,7 +16092,7 @@
       <c r="L27" s="117"/>
     </row>
     <row r="28" spans="1:12" ht="18.75">
-      <c r="A28" s="341" t="s">
+      <c r="A28" s="342" t="s">
         <v>1280</v>
       </c>
       <c r="B28" s="123" t="s">
@@ -16092,7 +16102,7 @@
         <v>1276</v>
       </c>
       <c r="D28" s="246"/>
-      <c r="E28" s="344" t="s">
+      <c r="E28" s="346" t="s">
         <v>1300</v>
       </c>
       <c r="F28" s="123" t="s">
@@ -16102,7 +16112,7 @@
         <v>956</v>
       </c>
       <c r="H28" s="246"/>
-      <c r="I28" s="344" t="s">
+      <c r="I28" s="346" t="s">
         <v>1300</v>
       </c>
       <c r="J28" s="123" t="s">
@@ -16114,7 +16124,7 @@
       <c r="L28" s="117"/>
     </row>
     <row r="29" spans="1:12" ht="18.75">
-      <c r="A29" s="342"/>
+      <c r="A29" s="343"/>
       <c r="B29" s="122" t="s">
         <v>1287</v>
       </c>
@@ -16122,7 +16132,7 @@
         <v>1277</v>
       </c>
       <c r="D29" s="248"/>
-      <c r="E29" s="345"/>
+      <c r="E29" s="347"/>
       <c r="F29" s="122" t="s">
         <v>931</v>
       </c>
@@ -16130,7 +16140,7 @@
         <v>957</v>
       </c>
       <c r="H29" s="246"/>
-      <c r="I29" s="345"/>
+      <c r="I29" s="347"/>
       <c r="J29" s="122" t="s">
         <v>1019</v>
       </c>
@@ -16140,7 +16150,7 @@
       <c r="L29" s="117"/>
     </row>
     <row r="30" spans="1:12" ht="18.75">
-      <c r="A30" s="342"/>
+      <c r="A30" s="343"/>
       <c r="B30" s="122" t="s">
         <v>1288</v>
       </c>
@@ -16148,13 +16158,13 @@
         <v>1278</v>
       </c>
       <c r="D30" s="248"/>
-      <c r="E30" s="345"/>
+      <c r="E30" s="347"/>
       <c r="F30" s="122" t="s">
         <v>1336</v>
       </c>
       <c r="G30" s="188"/>
       <c r="H30" s="246"/>
-      <c r="I30" s="345"/>
+      <c r="I30" s="347"/>
       <c r="J30" s="122" t="s">
         <v>1020</v>
       </c>
@@ -16164,7 +16174,7 @@
       <c r="L30" s="117"/>
     </row>
     <row r="31" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A31" s="343"/>
+      <c r="A31" s="344"/>
       <c r="B31" s="126" t="s">
         <v>1289</v>
       </c>
@@ -16172,13 +16182,13 @@
         <v>1279</v>
       </c>
       <c r="D31" s="248"/>
-      <c r="E31" s="346"/>
+      <c r="E31" s="348"/>
       <c r="F31" s="126" t="s">
         <v>1337</v>
       </c>
       <c r="G31" s="189"/>
       <c r="H31" s="246"/>
-      <c r="I31" s="346"/>
+      <c r="I31" s="348"/>
       <c r="J31" s="126" t="s">
         <v>1021</v>
       </c>
@@ -16188,7 +16198,7 @@
       <c r="L31" s="117"/>
     </row>
     <row r="32" spans="1:12" ht="18.75">
-      <c r="A32" s="354"/>
+      <c r="A32" s="345"/>
       <c r="B32" s="246"/>
       <c r="C32" s="248"/>
       <c r="D32" s="248"/>
@@ -16202,7 +16212,7 @@
       <c r="L32" s="117"/>
     </row>
     <row r="33" spans="1:12" ht="18.75">
-      <c r="A33" s="354"/>
+      <c r="A33" s="345"/>
       <c r="B33" s="246"/>
       <c r="C33" s="248"/>
       <c r="D33" s="248"/>
@@ -16216,7 +16226,7 @@
       <c r="L33" s="117"/>
     </row>
     <row r="34" spans="1:12" ht="18.75">
-      <c r="A34" s="354"/>
+      <c r="A34" s="345"/>
       <c r="B34" s="246"/>
       <c r="C34" s="248"/>
       <c r="D34" s="248"/>
@@ -16230,7 +16240,7 @@
       <c r="L34" s="117"/>
     </row>
     <row r="35" spans="1:12" ht="18.75">
-      <c r="A35" s="354"/>
+      <c r="A35" s="345"/>
       <c r="B35" s="246"/>
       <c r="C35" s="248"/>
       <c r="D35" s="248"/>
@@ -16244,7 +16254,7 @@
       <c r="L35" s="117"/>
     </row>
     <row r="36" spans="1:12" ht="18.75">
-      <c r="A36" s="354"/>
+      <c r="A36" s="345"/>
       <c r="B36" s="246"/>
       <c r="C36" s="248"/>
       <c r="D36" s="248"/>
@@ -16258,7 +16268,7 @@
       <c r="L36" s="117"/>
     </row>
     <row r="37" spans="1:12" ht="18.75">
-      <c r="A37" s="354"/>
+      <c r="A37" s="345"/>
       <c r="B37" s="246"/>
       <c r="C37" s="248"/>
       <c r="D37" s="248"/>
@@ -16272,7 +16282,7 @@
       <c r="L37" s="117"/>
     </row>
     <row r="38" spans="1:12" ht="18.75">
-      <c r="A38" s="354"/>
+      <c r="A38" s="345"/>
       <c r="B38" s="246"/>
       <c r="C38" s="248"/>
       <c r="D38" s="248"/>
@@ -16286,15 +16296,15 @@
       <c r="L38" s="117"/>
     </row>
     <row r="39" spans="1:12" ht="18.75">
-      <c r="A39" s="354"/>
+      <c r="A39" s="345"/>
       <c r="B39" s="246"/>
       <c r="C39" s="248"/>
       <c r="D39" s="248"/>
-      <c r="E39" s="353"/>
+      <c r="E39" s="341"/>
       <c r="F39" s="246"/>
       <c r="G39" s="246"/>
       <c r="H39" s="324"/>
-      <c r="I39" s="353"/>
+      <c r="I39" s="341"/>
       <c r="J39" s="246"/>
       <c r="K39" s="246"/>
       <c r="L39" s="117"/>
@@ -16304,11 +16314,11 @@
       <c r="B40" s="246"/>
       <c r="C40" s="247"/>
       <c r="D40" s="248"/>
-      <c r="E40" s="353"/>
+      <c r="E40" s="341"/>
       <c r="F40" s="246"/>
       <c r="G40" s="246"/>
       <c r="H40" s="324"/>
-      <c r="I40" s="353"/>
+      <c r="I40" s="341"/>
       <c r="J40" s="246"/>
       <c r="K40" s="246"/>
       <c r="L40" s="117"/>
@@ -16318,11 +16328,11 @@
       <c r="B41" s="246"/>
       <c r="C41" s="248"/>
       <c r="D41" s="248"/>
-      <c r="E41" s="353"/>
+      <c r="E41" s="341"/>
       <c r="F41" s="246"/>
       <c r="G41" s="246"/>
       <c r="H41" s="324"/>
-      <c r="I41" s="353"/>
+      <c r="I41" s="341"/>
       <c r="J41" s="246"/>
       <c r="K41" s="246"/>
       <c r="L41" s="117"/>
@@ -16332,11 +16342,11 @@
       <c r="B42" s="246"/>
       <c r="C42" s="248"/>
       <c r="D42" s="248"/>
-      <c r="E42" s="353"/>
+      <c r="E42" s="341"/>
       <c r="F42" s="246"/>
       <c r="G42" s="246"/>
       <c r="H42" s="324"/>
-      <c r="I42" s="353"/>
+      <c r="I42" s="341"/>
       <c r="J42" s="246"/>
       <c r="K42" s="246"/>
       <c r="L42" s="117"/>
@@ -16385,13 +16395,18 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="E39:E42"/>
-    <mergeCell ref="I39:I42"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A7"/>
     <mergeCell ref="I16:I19"/>
     <mergeCell ref="I12:I15"/>
     <mergeCell ref="I8:I11"/>
@@ -16402,18 +16417,13 @@
     <mergeCell ref="I28:I31"/>
     <mergeCell ref="E20:E23"/>
     <mergeCell ref="E24:E27"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="E39:E42"/>
+    <mergeCell ref="I39:I42"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="A36:A39"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -18331,54 +18341,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1">
-      <c r="A1" s="381" t="s">
+      <c r="A1" s="397" t="s">
         <v>1301</v>
       </c>
-      <c r="B1" s="382"/>
-      <c r="C1" s="382"/>
-      <c r="D1" s="382"/>
-      <c r="E1" s="382"/>
-      <c r="F1" s="382"/>
-      <c r="G1" s="382"/>
-      <c r="H1" s="383"/>
+      <c r="B1" s="398"/>
+      <c r="C1" s="398"/>
+      <c r="D1" s="398"/>
+      <c r="E1" s="398"/>
+      <c r="F1" s="398"/>
+      <c r="G1" s="398"/>
+      <c r="H1" s="399"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
-      <c r="A2" s="384"/>
-      <c r="B2" s="385"/>
-      <c r="C2" s="385"/>
-      <c r="D2" s="385"/>
-      <c r="E2" s="385"/>
-      <c r="F2" s="385"/>
-      <c r="G2" s="385"/>
-      <c r="H2" s="386"/>
+      <c r="A2" s="400"/>
+      <c r="B2" s="401"/>
+      <c r="C2" s="401"/>
+      <c r="D2" s="401"/>
+      <c r="E2" s="401"/>
+      <c r="F2" s="401"/>
+      <c r="G2" s="401"/>
+      <c r="H2" s="402"/>
     </row>
     <row r="3" spans="1:8" ht="23.25">
-      <c r="A3" s="387" t="s">
+      <c r="A3" s="403" t="s">
         <v>1129</v>
       </c>
-      <c r="B3" s="388"/>
-      <c r="C3" s="388"/>
-      <c r="D3" s="389"/>
-      <c r="E3" s="390" t="s">
+      <c r="B3" s="404"/>
+      <c r="C3" s="404"/>
+      <c r="D3" s="405"/>
+      <c r="E3" s="406" t="s">
         <v>1130</v>
       </c>
-      <c r="F3" s="388"/>
-      <c r="G3" s="388"/>
-      <c r="H3" s="391"/>
+      <c r="F3" s="404"/>
+      <c r="G3" s="404"/>
+      <c r="H3" s="407"/>
     </row>
     <row r="4" spans="1:8" ht="16.149999999999999" customHeight="1" thickBot="1">
-      <c r="A4" s="392" t="s">
+      <c r="A4" s="408" t="s">
         <v>1131</v>
       </c>
-      <c r="B4" s="393"/>
-      <c r="C4" s="393"/>
-      <c r="D4" s="394"/>
-      <c r="E4" s="395" t="s">
+      <c r="B4" s="409"/>
+      <c r="C4" s="409"/>
+      <c r="D4" s="410"/>
+      <c r="E4" s="411" t="s">
         <v>1132</v>
       </c>
-      <c r="F4" s="393"/>
-      <c r="G4" s="393"/>
-      <c r="H4" s="396"/>
+      <c r="F4" s="409"/>
+      <c r="G4" s="409"/>
+      <c r="H4" s="412"/>
     </row>
     <row r="5" spans="1:8" ht="19.5" thickBot="1">
       <c r="A5" s="196">
@@ -18857,12 +18867,12 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A25" s="378" t="s">
+      <c r="A25" s="394" t="s">
         <v>1149</v>
       </c>
-      <c r="B25" s="379"/>
-      <c r="C25" s="379"/>
-      <c r="D25" s="380"/>
+      <c r="B25" s="395"/>
+      <c r="C25" s="395"/>
+      <c r="D25" s="396"/>
       <c r="E25" s="197">
         <v>21</v>
       </c>
@@ -18877,14 +18887,14 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A26" s="403" t="s">
+      <c r="A26" s="384" t="s">
         <v>1122</v>
       </c>
-      <c r="B26" s="404"/>
-      <c r="C26" s="401" t="s">
+      <c r="B26" s="385"/>
+      <c r="C26" s="382" t="s">
         <v>1121</v>
       </c>
-      <c r="D26" s="402"/>
+      <c r="D26" s="383"/>
       <c r="E26" s="197">
         <v>22</v>
       </c>
@@ -18899,14 +18909,14 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A27" s="405" t="s">
+      <c r="A27" s="386" t="s">
         <v>1111</v>
       </c>
-      <c r="B27" s="406"/>
-      <c r="C27" s="409" t="s">
+      <c r="B27" s="387"/>
+      <c r="C27" s="390" t="s">
         <v>1304</v>
       </c>
-      <c r="D27" s="410"/>
+      <c r="D27" s="391"/>
       <c r="E27" s="197">
         <v>23</v>
       </c>
@@ -18921,14 +18931,14 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A28" s="405" t="s">
+      <c r="A28" s="386" t="s">
         <v>1116</v>
       </c>
-      <c r="B28" s="406"/>
-      <c r="C28" s="411" t="s">
+      <c r="B28" s="387"/>
+      <c r="C28" s="392" t="s">
         <v>1120</v>
       </c>
-      <c r="D28" s="412"/>
+      <c r="D28" s="393"/>
       <c r="E28" s="197">
         <v>24</v>
       </c>
@@ -18943,10 +18953,10 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A29" s="405" t="s">
+      <c r="A29" s="386" t="s">
         <v>374</v>
       </c>
-      <c r="B29" s="406"/>
+      <c r="B29" s="387"/>
       <c r="C29" s="300" t="s">
         <v>1310</v>
       </c>
@@ -18965,10 +18975,10 @@
       </c>
     </row>
     <row r="30" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A30" s="405" t="s">
+      <c r="A30" s="386" t="s">
         <v>365</v>
       </c>
-      <c r="B30" s="406"/>
+      <c r="B30" s="387"/>
       <c r="C30" s="300" t="s">
         <v>1311</v>
       </c>
@@ -18987,10 +18997,10 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A31" s="405" t="s">
+      <c r="A31" s="386" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="406"/>
+      <c r="B31" s="387"/>
       <c r="C31" s="300" t="s">
         <v>1312</v>
       </c>
@@ -19009,14 +19019,14 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A32" s="405" t="s">
+      <c r="A32" s="386" t="s">
         <v>188</v>
       </c>
-      <c r="B32" s="406"/>
-      <c r="C32" s="397" t="s">
+      <c r="B32" s="387"/>
+      <c r="C32" s="378" t="s">
         <v>1313</v>
       </c>
-      <c r="D32" s="398"/>
+      <c r="D32" s="379"/>
       <c r="E32" s="197">
         <v>28</v>
       </c>
@@ -19031,14 +19041,14 @@
       </c>
     </row>
     <row r="33" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A33" s="405" t="s">
+      <c r="A33" s="386" t="s">
         <v>1103</v>
       </c>
-      <c r="B33" s="406"/>
-      <c r="C33" s="397" t="s">
+      <c r="B33" s="387"/>
+      <c r="C33" s="378" t="s">
         <v>1314</v>
       </c>
-      <c r="D33" s="398"/>
+      <c r="D33" s="379"/>
       <c r="E33" s="197">
         <v>29</v>
       </c>
@@ -19053,14 +19063,14 @@
       </c>
     </row>
     <row r="34" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A34" s="407" t="s">
+      <c r="A34" s="388" t="s">
         <v>1100</v>
       </c>
-      <c r="B34" s="408"/>
-      <c r="C34" s="399" t="s">
+      <c r="B34" s="389"/>
+      <c r="C34" s="380" t="s">
         <v>1315</v>
       </c>
-      <c r="D34" s="400"/>
+      <c r="D34" s="381"/>
       <c r="E34" s="197">
         <v>30</v>
       </c>
@@ -19076,6 +19086,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="C34:D34"/>
@@ -19091,12 +19107,6 @@
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>